<commit_message>
leck eier, kb uf de kack
</commit_message>
<xml_diff>
--- a/M306_Projektplanung_Hunger_Weisshaar.xlsx
+++ b/M306_Projektplanung_Hunger_Weisshaar.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Auftragsplanung_mit_PM" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Auftragsplanung_mit_PM!$A$1:$L$37</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Auftragsplanung_mit_PM!$A$1:$L$38</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Auftragsplanung_mit_PM!$1:$1</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="107">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -316,7 +316,7 @@
     <t xml:space="preserve">M5</t>
   </si>
   <si>
-    <t xml:space="preserve">Abgabe PDF und Präsentation</t>
+    <t xml:space="preserve">Abgabe PDF</t>
   </si>
   <si>
     <t xml:space="preserve">0</t>
@@ -351,6 +351,9 @@
   <si>
     <t xml:space="preserve">Änderung 12.10.2026: Paket 3.1 am 12.10. (KW 42) von Lucas statt Nicolas durchgeführt; ChatGPT-Tageslimit erreicht (R1), P5/P6 mit zweitem Gratis-Konto nachgeholt.</t>
   </si>
+  <si>
+    <t xml:space="preserve">Stand 25.10.2026: Abgabetermin (M5) an die Vorgabe der Lehrperson angepasst: So 25.10.2026 statt Mi 21.10.2026; Präsentation nach der Abgabe.</t>
+  </si>
 </sst>
 </file>
 
@@ -358,7 +361,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="d&quot;. &quot;mmm"/>
+    <numFmt numFmtId="165" formatCode="[$-407]d&quot;. &quot;mmm"/>
     <numFmt numFmtId="166" formatCode="0.0#"/>
   </numFmts>
   <fonts count="8">
@@ -1803,7 +1806,7 @@
       <c r="J27" s="7"/>
       <c r="K27" s="7"/>
       <c r="L27" s="11" t="n">
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="M27" s="6"/>
       <c r="N27" s="6"/>
@@ -2103,7 +2106,9 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7"/>
-      <c r="B38" s="7"/>
+      <c r="B38" s="15" t="s">
+        <v>106</v>
+      </c>
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
@@ -25363,7 +25368,7 @@
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;CM306 – Projektplanung | Hunger, Weisshaar</oddHeader>
-    <oddFooter>&amp;LVersion 0.1 | 12.10.2026&amp;RSeite &amp;P von &amp;N</oddFooter>
+    <oddFooter>&amp;LVersion 1.0 | 25.10.2026&amp;RSeite &amp;P von &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>